<commit_message>
Strip letters from Order ProductID and Product short_code.
Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -815,7 +815,7 @@
   "StoreID": 1701,
   "SalesRepID": "THOMAS OUMA",
   "RouteID": 85,
-  "ProductID": "BIC976044",
+  "ProductID": "976044",
   "DistributorID": "???",
   "WarehouseID": 183,
   "OrderNumber": 60,
@@ -837,7 +837,7 @@
           <t>SHOP_ID -&gt; StoreID
 SALES_REP -&gt; SalesRepID
 ROUTEID -&gt; RouteID
-PRODUCT_CODE -&gt; ProductID
+PRODUCT_CODE -&gt; ProductID  (numeric part only)
 '' -&gt; DistributorID
 SUPPLIER_ID -&gt; WarehouseID
 ENTRY_ID -&gt; OrderNumber
@@ -928,7 +928,7 @@
   "product_name": "BIC",
   "ProductSKU": "CRISTAL MED BLU BX 25 BCL KE",
   "product_status": "Enabled",
-  "short_code": "BIC502418",
+  "short_code": "502418",
   "tax_code": "A",
   "hs_code": "",
   "focus_product": 0,
@@ -951,7 +951,7 @@
 product_name -&gt; product_name
 product_desc -&gt; ProductSKU
 product_status -&gt; product_status
-short_code -&gt; short_code
+short_code -&gt; short_code  (numeric part only)
 tax_code -&gt; tax_code
 hs_code -&gt; hs_code
 focus_product -&gt; focus_product
@@ -1886,7 +1886,7 @@
   "StoreID": 1701,
   "SalesRepID": "THOMAS OUMA",
   "RouteID": 85,
-  "ProductID": "BIC976044",
+  "ProductID": "976044",
   "DistributorID": "???",
   "WarehouseID": 183,
   "OrderNumber": 60,
@@ -1908,7 +1908,7 @@
           <t>SHOP_ID -&gt; StoreID
 SALES_REP -&gt; SalesRepID
 ROUTEID -&gt; RouteID
-PRODUCT_CODE -&gt; ProductID
+PRODUCT_CODE -&gt; ProductID  (numeric part only)
 '' -&gt; DistributorID
 SUPPLIER_ID -&gt; WarehouseID
 ENTRY_ID -&gt; OrderNumber
@@ -1999,7 +1999,7 @@
   "product_name": "BIC",
   "ProductSKU": "CRISTAL MED BLU BX 25 BCL KE",
   "product_status": "Enabled",
-  "short_code": "BIC502418",
+  "short_code": "502418",
   "tax_code": "A",
   "hs_code": "",
   "focus_product": 0,
@@ -2022,7 +2022,7 @@
 product_name -&gt; product_name
 product_desc -&gt; ProductSKU
 product_status -&gt; product_status
-short_code -&gt; short_code
+short_code -&gt; short_code  (numeric part only)
 tax_code -&gt; tax_code
 hs_code -&gt; hs_code
 focus_product -&gt; focus_product
@@ -3114,7 +3114,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>PRODUCT_CODE -&gt; ProductID</t>
+          <t>PRODUCT_CODE -&gt; ProductID  (numeric part only)</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>short_code -&gt; short_code</t>
+          <t>short_code -&gt; short_code  (numeric part only)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Put Exp, PAPI, and SAPI for every environment in one Postman collection.
Local, Sandbox, Presandbox, and Production are folders in the same collection. PAPI still sends a hardcoded Authorization header.

Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -4662,12 +4662,24 @@
           <t>presandbox</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>(set on the Presandbox folder)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>(set on the Presandbox folder)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>(set on the Presandbox folder)</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Paste hosts when the presandbox apps are deployed. Collection uses {{exp_base}} / {{papi_base}} / {{sapi_base}}.</t>
+          <t>One Postman collection. Open the Presandbox folder and paste the three hosts on that folder.</t>
         </is>
       </c>
     </row>
@@ -4677,12 +4689,24 @@
           <t>production</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr"/>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>(set on the Production folder)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>(set on the Production folder)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>(set on the Production folder)</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Paste hosts when the production apps are deployed.</t>
+          <t>One Postman collection. Open the Production folder and paste the three hosts on that folder.</t>
         </is>
       </c>
     </row>
@@ -4821,7 +4845,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Import matching Postman environment</t>
+          <t>Folders inside the single Postman collection</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Kenya guide and Excel for 2000-row pages and new sample payloads.
Set page size to 2000, restore a bold Confidential v1.0 page footer, drop Country, use the token URL in credentials, and refresh Invoice/Order/Product/Stock samples.

Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
+++ b/mapping/SAT-Datashare-SAPI-PAPI-EAPI-payloads.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Payloads" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Endpoints" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Current field map" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Query parameters" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Authentication" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Environments" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="How this sheet is filled" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payloads" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Endpoints" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current field map" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Query parameters" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Authentication" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environments" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How this sheet is filled" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Payloads'!$A$1:$J$9</definedName>
@@ -3693,7 +3693,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 10000.</t>
+          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 2000.</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3789,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 10000.</t>
+          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 2000.</t>
         </is>
       </c>
     </row>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 10000.</t>
+          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 2000.</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 10000.</t>
+          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 2000.</t>
         </is>
       </c>
     </row>
@@ -4077,7 +4077,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 10000.</t>
+          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 2000.</t>
         </is>
       </c>
     </row>
@@ -4173,7 +4173,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 10000.</t>
+          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 2000.</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 10000.</t>
+          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 2000.</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4365,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 10000.</t>
+          <t>database = MySQL schema. supplier = products.supplier. pageNumber 0-based. page size 2000.</t>
         </is>
       </c>
     </row>

</xml_diff>